<commit_message>
SEASON 2 STATS UPDATE
</commit_message>
<xml_diff>
--- a/docs/stats.xlsx
+++ b/docs/stats.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\marc\GitHub\304-game\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B9A7D97-2F05-469D-BAFA-CF40FB7BDA55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226B2D8F-8E9C-4084-98E0-13FC6F7DBC2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="103">
   <si>
     <t>Date</t>
   </si>
@@ -368,6 +368,12 @@
   </si>
   <si>
     <t>R20260529-1</t>
+  </si>
+  <si>
+    <t>SEASON 2 START</t>
+  </si>
+  <si>
+    <t>R20260725-1</t>
   </si>
 </sst>
 </file>
@@ -797,7 +803,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.90625" customWidth="1"/>
@@ -958,7 +964,7 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="E3" s="3">
-        <f t="shared" ref="E3:E31" si="1">MOD(D3 - C3, 1)</f>
+        <f t="shared" ref="E3:E32" si="1">MOD(D3 - C3, 1)</f>
         <v>0.16666666666666663</v>
       </c>
       <c r="F3" t="str" cm="1">
@@ -3487,7 +3493,7 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" t="str">
-        <f t="shared" ref="A29:A31" si="3">"R"&amp;TEXT(B29,"yyyymmdd")&amp;"-"&amp;COUNTIFS($B:$B,B29,$C:$C,"&lt;="&amp;C29)</f>
+        <f t="shared" ref="A29:A32" si="3">"R"&amp;TEXT(B29,"yyyymmdd")&amp;"-"&amp;COUNTIFS($B:$B,B29,$C:$C,"&lt;="&amp;C29)</f>
         <v>R20260427-1</v>
       </c>
       <c r="B29" s="1">
@@ -3773,8 +3779,107 @@
         <v>0 (20)</v>
       </c>
     </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A32" t="str">
+        <f t="shared" si="3"/>
+        <v>R20260725-1</v>
+      </c>
+      <c r="B32" s="1">
+        <v>46228</v>
+      </c>
+      <c r="C32" s="2">
+        <v>12</v>
+      </c>
+      <c r="E32" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F32" t="str" cm="1">
+        <f t="array" ref="F32">COUNTIFS(
+ Matches!$A$2:$A$200,$A32,
+ Matches!$I$2:$I$200,"*"&amp;F$1&amp;"*"
+)
+&amp;" ("&amp;
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A32) *
+ ((Matches!$C$2:$C$200=F$1)+(Matches!$D$2:$D$200=F$1)) *
+ Matches!$G$2:$G$200
+)
++
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A32) *
+ ((Matches!$E$2:$E$200=F$1)+(Matches!$F$2:$F$200=F$1)) *
+ Matches!$H$2:$H$200
+)
+&amp;")"</f>
+        <v>2 (27)</v>
+      </c>
+      <c r="G32" t="str" cm="1">
+        <f t="array" ref="G32">COUNTIFS(
+ Matches!$A$2:$A$200,$A32,
+ Matches!$I$2:$I$200,"*"&amp;G$1&amp;"*"
+)
+&amp;" ("&amp;
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A32) *
+ ((Matches!$C$2:$C$200=G$1)+(Matches!$D$2:$D$200=G$1)) *
+ Matches!$G$2:$G$200
+)
++
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A32) *
+ ((Matches!$E$2:$E$200=G$1)+(Matches!$F$2:$F$200=G$1)) *
+ Matches!$H$2:$H$200
+)
+&amp;")"</f>
+        <v>2 (26)</v>
+      </c>
+      <c r="H32" t="str" cm="1">
+        <f t="array" ref="H32">COUNTIFS(
+ Matches!$A$2:$A$200,$A32,
+ Matches!$I$2:$I$200,"*"&amp;H$1&amp;"*"
+)
+&amp;" ("&amp;
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A32) *
+ ((Matches!$C$2:$C$200=H$1)+(Matches!$D$2:$D$200=H$1)) *
+ Matches!$G$2:$G$200
+)
++
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A32) *
+ ((Matches!$E$2:$E$200=H$1)+(Matches!$F$2:$F$200=H$1)) *
+ Matches!$H$2:$H$200
+)
+&amp;")"</f>
+        <v>2 (26)</v>
+      </c>
+      <c r="I32" t="str" cm="1">
+        <f t="array" ref="I32">COUNTIFS(
+ Matches!$A$2:$A$200,$A32,
+ Matches!$I$2:$I$200,"*"&amp;I$1&amp;"*"
+)
+&amp;" ("&amp;
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A32) *
+ ((Matches!$C$2:$C$200=I$1)+(Matches!$D$2:$D$200=I$1)) *
+ Matches!$G$2:$G$200
+)
++
+SUMPRODUCT(
+ (Matches!$A$2:$A$200=$A32) *
+ ((Matches!$E$2:$E$200=I$1)+(Matches!$F$2:$F$200=I$1)) *
+ Matches!$H$2:$H$200
+)
+&amp;")"</f>
+        <v>0 (19)</v>
+      </c>
+      <c r="J32" t="s">
+        <v>101</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:I31">
+  <conditionalFormatting sqref="F2:I32">
     <cfRule type="expression" dxfId="10" priority="1">
       <formula>LEFT(F2,1)="0"</formula>
     </cfRule>
@@ -3805,7 +3910,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B6F95CC-DDBC-4D0D-92B0-0E6D3AF66C09}">
-  <dimension ref="A1:K90"/>
+  <dimension ref="A1:K93"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.90625" customWidth="1"/>
@@ -3919,7 +4024,7 @@
         <v>10</v>
       </c>
       <c r="I3" t="str">
-        <f t="shared" ref="I3:I90" si="0">IF(G3&gt;H3,
+        <f t="shared" ref="I3:I93" si="0">IF(G3&gt;H3,
    IF(C3&lt;D3, C3&amp;"/"&amp;D3, D3&amp;"/"&amp;C3),
    IF(E3&lt;F3, E3&amp;"/"&amp;F3, F3&amp;"/"&amp;E3)
 )</f>
@@ -6193,7 +6298,7 @@
         <v>ML/MN</v>
       </c>
       <c r="K67" t="str">
-        <f t="shared" ref="K67:K90" si="2">_xlfn.CONCAT(A67, "-", B67)</f>
+        <f t="shared" ref="K67:K93" si="2">_xlfn.CONCAT(A67, "-", B67)</f>
         <v>R20260318-3-1</v>
       </c>
     </row>
@@ -6989,6 +7094,108 @@
       <c r="K90" t="str">
         <f t="shared" si="2"/>
         <v>R20260529-1-3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>102</v>
+      </c>
+      <c r="B91">
+        <v>1</v>
+      </c>
+      <c r="C91" t="s">
+        <v>13</v>
+      </c>
+      <c r="D91" t="s">
+        <v>15</v>
+      </c>
+      <c r="E91" t="s">
+        <v>12</v>
+      </c>
+      <c r="F91" t="s">
+        <v>14</v>
+      </c>
+      <c r="G91" s="4">
+        <v>6</v>
+      </c>
+      <c r="H91" s="4">
+        <v>10</v>
+      </c>
+      <c r="I91" t="str">
+        <f t="shared" si="0"/>
+        <v>LX/MN</v>
+      </c>
+      <c r="K91" t="str">
+        <f t="shared" si="2"/>
+        <v>R20260725-1-1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>102</v>
+      </c>
+      <c r="B92">
+        <v>2</v>
+      </c>
+      <c r="C92" t="s">
+        <v>13</v>
+      </c>
+      <c r="D92" t="s">
+        <v>12</v>
+      </c>
+      <c r="E92" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" t="s">
+        <v>15</v>
+      </c>
+      <c r="G92" s="4">
+        <v>7</v>
+      </c>
+      <c r="H92" s="4">
+        <v>10</v>
+      </c>
+      <c r="I92" t="str">
+        <f t="shared" si="0"/>
+        <v>ML/MN</v>
+      </c>
+      <c r="K92" t="str">
+        <f t="shared" si="2"/>
+        <v>R20260725-1-2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>102</v>
+      </c>
+      <c r="B93">
+        <v>3</v>
+      </c>
+      <c r="C93" t="s">
+        <v>14</v>
+      </c>
+      <c r="D93" t="s">
+        <v>13</v>
+      </c>
+      <c r="E93" t="s">
+        <v>12</v>
+      </c>
+      <c r="F93" t="s">
+        <v>15</v>
+      </c>
+      <c r="G93" s="4">
+        <v>6</v>
+      </c>
+      <c r="H93" s="4">
+        <v>10</v>
+      </c>
+      <c r="I93" t="str">
+        <f t="shared" si="0"/>
+        <v>LX/ML</v>
+      </c>
+      <c r="K93" t="str">
+        <f t="shared" si="2"/>
+        <v>R20260725-1-3</v>
       </c>
     </row>
   </sheetData>
@@ -8547,15 +8754,15 @@
     )
   )
 )</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" cm="1">
         <f t="array" aca="1" ref="D2" ca="1">SUMPRODUCT(--LEFT(INDIRECT("Revolutions!F2:F"&amp;$G$2)))</f>
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E2" cm="1">
         <f t="array" aca="1" ref="E2" ca="1">SUMPRODUCT(--MID(INDIRECT("Revolutions!F2:F"&amp;$G$2), FIND("(",INDIRECT("Revolutions!F2:F"&amp;$G$2))+1, LEN(INDIRECT("Revolutions!F2:F"&amp;$G$2))-FIND("(",INDIRECT("Revolutions!F2:F"&amp;$G$2))-1))</f>
-        <v>669</v>
+        <v>696</v>
       </c>
       <c r="F2" cm="1">
         <f t="array" aca="1" ref="F2" ca="1">SUM(
@@ -8571,11 +8778,11 @@
   )
  )
 )</f>
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G2" cm="1">
         <f t="array" ref="G2">MATCH(2,1/(Revolutions!A:A&lt;&gt;""),1)</f>
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -8609,11 +8816,11 @@
       </c>
       <c r="D3" cm="1">
         <f t="array" aca="1" ref="D3" ca="1">SUMPRODUCT(--LEFT(INDIRECT("Revolutions!G2:G"&amp;$G$2),1))</f>
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E3" cm="1">
         <f t="array" aca="1" ref="E3" ca="1">SUMPRODUCT(--MID(INDIRECT("Revolutions!G2:G"&amp;$G$2), FIND("(",INDIRECT("Revolutions!G2:G"&amp;$G$2))+1, LEN(INDIRECT("Revolutions!G2:G"&amp;$G$2))-FIND("(",INDIRECT("Revolutions!G2:G"&amp;$G$2))-1))</f>
-        <v>681</v>
+        <v>707</v>
       </c>
       <c r="F3" cm="1">
         <f t="array" aca="1" ref="F3" ca="1">SUM(
@@ -8629,7 +8836,7 @@
   )
  )
 )</f>
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -8663,11 +8870,11 @@
       </c>
       <c r="D4" cm="1">
         <f t="array" aca="1" ref="D4" ca="1">SUMPRODUCT(--LEFT(INDIRECT("Revolutions!H2:H"&amp;$G$2)))</f>
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E4" cm="1">
         <f t="array" aca="1" ref="E4" ca="1">SUMPRODUCT(--MID(INDIRECT("Revolutions!H2:H"&amp;$G$2), FIND("(",INDIRECT("Revolutions!H2:H"&amp;$G$2))+1, LEN(INDIRECT("Revolutions!H2:H"&amp;$G$2))-FIND("(",INDIRECT("Revolutions!H2:H"&amp;$G$2))-1))</f>
-        <v>711</v>
+        <v>737</v>
       </c>
       <c r="F4" cm="1">
         <f t="array" aca="1" ref="F4" ca="1">SUM(
@@ -8683,7 +8890,7 @@
   )
  )
 )</f>
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -8721,7 +8928,7 @@
       </c>
       <c r="E5" cm="1">
         <f t="array" aca="1" ref="E5" ca="1">SUMPRODUCT(--MID(INDIRECT("Revolutions!I2:I"&amp;$G$2), FIND("(",INDIRECT("Revolutions!I2:I"&amp;$G$2))+1, LEN(INDIRECT("Revolutions!I2:I"&amp;$G$2))-FIND("(",INDIRECT("Revolutions!I2:I"&amp;$G$2))-1))</f>
-        <v>639</v>
+        <v>658</v>
       </c>
       <c r="F5" cm="1">
         <f t="array" aca="1" ref="F5" ca="1">SUM(
@@ -8737,7 +8944,7 @@
   )
  )
 )</f>
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>